<commit_message>
docs: update Management Interfaces Matrix on all tabs (Overview, Matrix, ViewModel Usage, CQRS Handler Usage, Sources, Legend) to reflect CHAT-001/CONN-001 CQRS remediation (0 logic offenses for Chat/Connection ViewModels; added handlers)
</commit_message>
<xml_diff>
--- a/docs/McpServerManager_Management_Interfaces_Matrix.xlsx
+++ b/docs/McpServerManager_Management_Interfaces_Matrix.xlsx
@@ -652,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -675,7 +675,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-26T19:34:19.410161 | Agent: GrokCode | Workspace: McpServerManager | MCP: http://PAYTON-LEGION2:7147</t>
+          <t>Generated: 2026-06-26T19:34:19.410161 | Updated: 2026-07-01 | Agent: GrokCode | CONN-001 + CHAT-001: ChatWindowViewModel, ConnectionViewModel now use CQRS dispatch (0 logic offenses)</t>
         </is>
       </c>
     </row>
@@ -764,6 +764,13 @@
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>MCP TODOs (via /mcpserver/todo): ARCH-WORKSPACEEDIT-*, PLAN-REQSDESKTOP-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Remediation: ViewModels migrated to dispatch (FetchMcpApiKeyCommand etc). Per-file gates passed. See ViewModel Usage and CQRS Handler Usage tabs.</t>
         </is>
       </c>
     </row>
@@ -1054,12 +1061,12 @@
       </c>
       <c r="H7" s="38" t="inlineStr">
         <is>
-          <t>Partial (uses core ones: Todo, Workspace, Voice, Connection, Chat, Log)</t>
+          <t>Full (uses shared UI.Core: Todo, Workspace, Voice, Connection, ChatWindow, Log + new CQRS dispatch for auth)</t>
         </is>
       </c>
       <c r="I7" s="38" t="inlineStr">
         <is>
-          <t>Partial (uses many shared handlers via McpHost)</t>
+          <t>Full (uses shared UI.Core handlers + Connection auth commands: FetchMcpApiKey, Logout etc.)</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
@@ -1121,12 +1128,12 @@
       </c>
       <c r="H8" s="38" t="inlineStr">
         <is>
-          <t>Partial (similar to Desktop + mobile specific)</t>
+          <t>Full (uses shared UI.Core: Todo, Workspace, Voice, Connection, Chat, Log + CQRS remediation)</t>
         </is>
       </c>
       <c r="I8" s="38" t="inlineStr">
         <is>
-          <t>Partial (uses many shared handlers)</t>
+          <t>Full (shared handlers + Connection CQRS dispatch)</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -1311,7 +1318,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>State Legend &amp; Color Key</t>
+          <t>State Legend &amp; Color Key (Updated 2026-07-01)</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1545,6 +1552,13 @@
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Session Log: GrokCode-20260627T000145Z-agents-md-repl (audit turn req-20260627T003500Z-audit-matrix-001 + save turn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-01: CONN-001 remediation - ConnectionViewModel now fully dispatches CQRS (no direct auth service logic). ChatWindow also clean. See updated ViewModel Usage and CQRS Handler Usage.</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1583,7 +1597,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-26T19:43:06.672633 | Green = Shared (UI.Core) | Red = Proprietary | ✓ = Used by app</t>
+          <t>Updated 2026-07-01 | ChatWindowViewModel &amp; ConnectionViewModel remediated to 0 logic offenses via CQRS dispatch (CONN-001 + CHAT-001)</t>
         </is>
       </c>
     </row>
@@ -1875,10 +1889,10 @@
         </is>
       </c>
       <c r="H13" s="41" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I13" s="42" t="n">
-        <v>0.2803030303030303</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1933,10 +1947,10 @@
         </is>
       </c>
       <c r="H15" s="41" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="I15" s="42" t="n">
-        <v>0.2994505494505494</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3593,15 +3607,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
   </sheetData>
   <autoFilter ref="A4:I77"/>
   <mergeCells count="3">
@@ -3641,7 +3646,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-26T19:44:31.950696 | Green rows = Shared (UI.Core/Handlers) | Red = Proprietary | ✓ = Handler used/registered by the app</t>
+          <t>Generated: 2026-06-26T19:44:31.950696 | Updated 2026-07-01 for CHAT+CONN CQRS (new auth handlers)</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5229,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>Shared handlers live in McpServerManager.UI.Core/Handlers/*.cs and are wired via McpHostBuilderExtensions + host service registrations. Proprietary handlers are defined per-app (e.g. Director-specific dialogs).</t>
+          <t>Shared handlers live in McpServerManager.UI.Core/Handlers/*.cs and are wired via McpHostBuilderExtensions + host service registrations. Proprietary handlers are defined per-app (e.g. Director-specific dialogs). | 2026-07-01: Added FetchMcpApiKeyCommandHandler, LogoutCommandHandler, ProbeHealthAndResolveUrlQueryHandler, StartDeviceAuthorizationCommandHandler, PollForAccessTokenCommandHandler (CONN-001)</t>
         </is>
       </c>
     </row>

</xml_diff>